<commit_message>
WAWI.OL STD, PP&E + Excel
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/WAWI.OL.xlsx
+++ b/data/obx_xlsx/WAWI.OL.xlsx
@@ -10498,8 +10498,14 @@
       <c r="P64" s="15">
         <v>10345.49</v>
       </c>
-      <c r="Q64" s="15"/>
-      <c r="R64" s="15"/>
+      <c r="Q64" s="23">
+        <f>Q68+Q72</f>
+        <v>6520.41</v>
+      </c>
+      <c r="R64" s="23">
+        <f>R73+R79</f>
+        <v>6870.98</v>
+      </c>
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="14" t="s">

</xml_diff>